<commit_message>
Add sale branch to membership and services exports
</commit_message>
<xml_diff>
--- a/output/20260630_delivery_without_active_problems/problem_1_no_payment_cash_3_cases_20260630.xlsx
+++ b/output/20260630_delivery_without_active_problems/problem_1_no_payment_cash_3_cases_20260630.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Импорт_абонементы" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Импорт_абонементы'!$A$1:$U$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Импорт_абонементы'!$A$1:$V$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -459,6 +459,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
     <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -567,6 +568,11 @@
           <t>manager</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>филиал</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -638,6 +644,11 @@
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Васильева Яна Денисовна</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Фитнес Империя (Гоголевский)</t>
         </is>
       </c>
     </row>
@@ -715,6 +726,11 @@
           <t>Соколова Анастасия Александровна</t>
         </is>
       </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Фитнес Империя (Гоголевский)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
@@ -790,9 +806,14 @@
           <t>Петрова Полина Владимировна</t>
         </is>
       </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Фитнес Империя (Гоголевский)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U4"/>
+  <autoFilter ref="A1:V4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>